<commit_message>
updating bootstrapped estimates to 1000 instead of 100. Still tinkering with permutation test as I can't get it quite correct.
</commit_message>
<xml_diff>
--- a/data/crit_values_final.xlsx
+++ b/data/crit_values_final.xlsx
@@ -178,19 +178,19 @@
         <v>12</v>
       </c>
       <c r="B2" t="n">
-        <v>43.7</v>
+        <v>43.2</v>
       </c>
       <c r="C2" t="n">
-        <v>47.6</v>
+        <v>47.3</v>
       </c>
       <c r="D2" t="n">
         <v>51.1</v>
       </c>
       <c r="E2" t="n">
-        <v>50.9</v>
+        <v>50.5</v>
       </c>
       <c r="F2" t="n">
-        <v>51.9</v>
+        <v>51.8</v>
       </c>
       <c r="G2" t="n">
         <v>52.5</v>
@@ -199,10 +199,10 @@
         <v>53.4</v>
       </c>
       <c r="I2" t="n">
-        <v>55.6</v>
+        <v>55.7</v>
       </c>
       <c r="J2" t="n">
-        <v>58.4</v>
+        <v>58.9</v>
       </c>
       <c r="K2" t="n" s="2">
         <v>44733.0</v>
@@ -216,31 +216,31 @@
         <v>13</v>
       </c>
       <c r="B3" t="n">
-        <v>42.3</v>
+        <v>41.3</v>
       </c>
       <c r="C3" t="n">
-        <v>45.1</v>
+        <v>44.8</v>
       </c>
       <c r="D3" t="n">
-        <v>47.9</v>
+        <v>47.7</v>
       </c>
       <c r="E3" t="n">
-        <v>51.2</v>
+        <v>51.1</v>
       </c>
       <c r="F3" t="n">
-        <v>52.1</v>
+        <v>52.2</v>
       </c>
       <c r="G3" t="n">
-        <v>53.2</v>
+        <v>53.7</v>
       </c>
       <c r="H3" t="n">
-        <v>55.3</v>
+        <v>55.0</v>
       </c>
       <c r="I3" t="n">
-        <v>58.4</v>
+        <v>58.8</v>
       </c>
       <c r="J3" t="n">
-        <v>62.0</v>
+        <v>63.5</v>
       </c>
       <c r="K3" t="n" s="2">
         <v>44733.0</v>
@@ -260,10 +260,10 @@
         <v>44.3</v>
       </c>
       <c r="D4" t="n">
-        <v>47.0</v>
+        <v>46.7</v>
       </c>
       <c r="E4" t="n">
-        <v>50.9</v>
+        <v>50.8</v>
       </c>
       <c r="F4" t="n">
         <v>51.9</v>
@@ -272,13 +272,13 @@
         <v>53.5</v>
       </c>
       <c r="H4" t="n">
-        <v>54.4</v>
+        <v>54.7</v>
       </c>
       <c r="I4" t="n">
         <v>58.7</v>
       </c>
       <c r="J4" t="n">
-        <v>62.7</v>
+        <v>62.9</v>
       </c>
       <c r="K4" t="n" s="2">
         <v>44733.0</v>
@@ -292,13 +292,13 @@
         <v>15</v>
       </c>
       <c r="B5" t="n">
-        <v>40.3</v>
+        <v>39.8</v>
       </c>
       <c r="C5" t="n">
-        <v>42.4</v>
+        <v>42.5</v>
       </c>
       <c r="D5" t="n">
-        <v>44.7</v>
+        <v>45.2</v>
       </c>
       <c r="E5" t="n">
         <v>50.9</v>
@@ -307,16 +307,16 @@
         <v>52.0</v>
       </c>
       <c r="G5" t="n">
-        <v>53.2</v>
+        <v>53.3</v>
       </c>
       <c r="H5" t="n">
-        <v>57.2</v>
+        <v>57.0</v>
       </c>
       <c r="I5" t="n">
-        <v>60.5</v>
+        <v>60.4</v>
       </c>
       <c r="J5" t="n">
-        <v>64.1</v>
+        <v>63.9</v>
       </c>
       <c r="K5" t="n" s="2">
         <v>44733.0</v>
@@ -336,10 +336,10 @@
         <v>43.5</v>
       </c>
       <c r="D6" t="n">
-        <v>47.4</v>
+        <v>47.2</v>
       </c>
       <c r="E6" t="n">
-        <v>51.2</v>
+        <v>51.0</v>
       </c>
       <c r="F6" t="n">
         <v>52.4</v>
@@ -348,13 +348,13 @@
         <v>54.1</v>
       </c>
       <c r="H6" t="n">
-        <v>56.9</v>
+        <v>56.2</v>
       </c>
       <c r="I6" t="n">
-        <v>60.5</v>
+        <v>60.3</v>
       </c>
       <c r="J6" t="n">
-        <v>63.4</v>
+        <v>64.3</v>
       </c>
       <c r="K6" t="n" s="2">
         <v>44733.0</v>
@@ -368,31 +368,31 @@
         <v>17</v>
       </c>
       <c r="B7" t="n">
-        <v>40.8</v>
+        <v>40.3</v>
       </c>
       <c r="C7" t="n">
-        <v>43.5</v>
+        <v>43.4</v>
       </c>
       <c r="D7" t="n">
-        <v>46.5</v>
+        <v>46.7</v>
       </c>
       <c r="E7" t="n">
         <v>49.7</v>
       </c>
       <c r="F7" t="n">
-        <v>50.7</v>
+        <v>50.8</v>
       </c>
       <c r="G7" t="n">
-        <v>52.0</v>
+        <v>52.2</v>
       </c>
       <c r="H7" t="n">
         <v>53.7</v>
       </c>
       <c r="I7" t="n">
-        <v>57.2</v>
+        <v>57.3</v>
       </c>
       <c r="J7" t="n">
-        <v>61.8</v>
+        <v>61.7</v>
       </c>
       <c r="K7" t="n" s="2">
         <v>44733.0</v>
@@ -406,13 +406,13 @@
         <v>18</v>
       </c>
       <c r="B8" t="n">
-        <v>41.8</v>
+        <v>42.3</v>
       </c>
       <c r="C8" t="n">
-        <v>44.4</v>
+        <v>44.5</v>
       </c>
       <c r="D8" t="n">
-        <v>47.0</v>
+        <v>46.7</v>
       </c>
       <c r="E8" t="n">
         <v>50.0</v>
@@ -421,16 +421,16 @@
         <v>51.0</v>
       </c>
       <c r="G8" t="n">
-        <v>52.1</v>
+        <v>52.2</v>
       </c>
       <c r="H8" t="n">
-        <v>52.7</v>
+        <v>53.2</v>
       </c>
       <c r="I8" t="n">
         <v>56.7</v>
       </c>
       <c r="J8" t="n">
-        <v>60.2</v>
+        <v>60.4</v>
       </c>
       <c r="K8" t="n" s="2">
         <v>44733.0</v>
@@ -444,31 +444,31 @@
         <v>19</v>
       </c>
       <c r="B9" t="n">
-        <v>40.0</v>
+        <v>40.3</v>
       </c>
       <c r="C9" t="n">
-        <v>42.8</v>
+        <v>42.6</v>
       </c>
       <c r="D9" t="n">
-        <v>45.5</v>
+        <v>45.2</v>
       </c>
       <c r="E9" t="n">
-        <v>50.7</v>
+        <v>50.6</v>
       </c>
       <c r="F9" t="n">
-        <v>51.5</v>
+        <v>51.6</v>
       </c>
       <c r="G9" t="n">
-        <v>52.3</v>
+        <v>52.5</v>
       </c>
       <c r="H9" t="n">
-        <v>56.9</v>
+        <v>57.2</v>
       </c>
       <c r="I9" t="n">
-        <v>59.6</v>
+        <v>59.9</v>
       </c>
       <c r="J9" t="n">
-        <v>62.0</v>
+        <v>62.4</v>
       </c>
       <c r="K9" t="n" s="2">
         <v>44733.0</v>
@@ -488,25 +488,25 @@
         <v>46.5</v>
       </c>
       <c r="D10" t="n">
-        <v>48.4</v>
+        <v>48.7</v>
       </c>
       <c r="E10" t="n">
         <v>52.8</v>
       </c>
       <c r="F10" t="n">
-        <v>54.1</v>
+        <v>53.9</v>
       </c>
       <c r="G10" t="n">
-        <v>55.1</v>
+        <v>55.2</v>
       </c>
       <c r="H10" t="n">
-        <v>58.4</v>
+        <v>57.8</v>
       </c>
       <c r="I10" t="n">
-        <v>61.0</v>
+        <v>60.8</v>
       </c>
       <c r="J10" t="n">
-        <v>63.2</v>
+        <v>63.6</v>
       </c>
       <c r="K10" t="n" s="2">
         <v>44733.0</v>
@@ -520,31 +520,31 @@
         <v>21</v>
       </c>
       <c r="B11" t="n">
-        <v>40.0</v>
+        <v>39.8</v>
       </c>
       <c r="C11" t="n">
-        <v>43.7</v>
+        <v>44.0</v>
       </c>
       <c r="D11" t="n">
-        <v>47.7</v>
+        <v>48.2</v>
       </c>
       <c r="E11" t="n">
-        <v>52.3</v>
+        <v>51.9</v>
       </c>
       <c r="F11" t="n">
-        <v>53.4</v>
+        <v>53.5</v>
       </c>
       <c r="G11" t="n">
-        <v>54.9</v>
+        <v>55.2</v>
       </c>
       <c r="H11" t="n">
         <v>58.6</v>
       </c>
       <c r="I11" t="n">
-        <v>62.3</v>
+        <v>62.2</v>
       </c>
       <c r="J11" t="n">
-        <v>66.5</v>
+        <v>65.9</v>
       </c>
       <c r="K11" t="n" s="2">
         <v>44733.0</v>
@@ -558,31 +558,31 @@
         <v>22</v>
       </c>
       <c r="B12" t="n">
-        <v>34.1</v>
+        <v>34.8</v>
       </c>
       <c r="C12" t="n">
-        <v>40.3</v>
+        <v>40.6</v>
       </c>
       <c r="D12" t="n">
         <v>46.2</v>
       </c>
       <c r="E12" t="n">
-        <v>47.3</v>
+        <v>47.2</v>
       </c>
       <c r="F12" t="n">
         <v>48.9</v>
       </c>
       <c r="G12" t="n">
-        <v>50.2</v>
+        <v>50.7</v>
       </c>
       <c r="H12" t="n">
-        <v>51.6</v>
+        <v>51.7</v>
       </c>
       <c r="I12" t="n">
-        <v>56.6</v>
+        <v>56.5</v>
       </c>
       <c r="J12" t="n">
-        <v>60.3</v>
+        <v>60.9</v>
       </c>
       <c r="K12" t="n" s="2">
         <v>44733.0</v>
@@ -599,13 +599,13 @@
         <v>43.2</v>
       </c>
       <c r="C13" t="n">
-        <v>46.0</v>
+        <v>46.1</v>
       </c>
       <c r="D13" t="n">
         <v>49.2</v>
       </c>
       <c r="E13" t="n">
-        <v>51.4</v>
+        <v>51.3</v>
       </c>
       <c r="F13" t="n">
         <v>52.5</v>
@@ -614,13 +614,13 @@
         <v>54.2</v>
       </c>
       <c r="H13" t="n">
-        <v>54.2</v>
+        <v>54.1</v>
       </c>
       <c r="I13" t="n">
-        <v>58.4</v>
+        <v>58.2</v>
       </c>
       <c r="J13" t="n">
-        <v>62.3</v>
+        <v>62.8</v>
       </c>
       <c r="K13" t="n" s="2">
         <v>44768.0</v>
@@ -634,10 +634,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>45.4</v>
+        <v>45.7</v>
       </c>
       <c r="C14" t="n">
-        <v>47.8</v>
+        <v>47.9</v>
       </c>
       <c r="D14" t="n">
         <v>49.7</v>
@@ -649,16 +649,16 @@
         <v>53.2</v>
       </c>
       <c r="G14" t="n">
-        <v>54.4</v>
+        <v>54.5</v>
       </c>
       <c r="H14" t="n">
         <v>54.9</v>
       </c>
       <c r="I14" t="n">
-        <v>57.8</v>
+        <v>57.9</v>
       </c>
       <c r="J14" t="n">
-        <v>62.0</v>
+        <v>61.9</v>
       </c>
       <c r="K14" t="n" s="2">
         <v>44768.0</v>
@@ -672,19 +672,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>45.0</v>
+        <v>45.2</v>
       </c>
       <c r="C15" t="n">
-        <v>47.8</v>
+        <v>47.9</v>
       </c>
       <c r="D15" t="n">
         <v>50.2</v>
       </c>
       <c r="E15" t="n">
-        <v>51.7</v>
+        <v>51.8</v>
       </c>
       <c r="F15" t="n">
-        <v>52.7</v>
+        <v>52.8</v>
       </c>
       <c r="G15" t="n">
         <v>54.1</v>
@@ -693,7 +693,7 @@
         <v>54.6</v>
       </c>
       <c r="I15" t="n">
-        <v>57.2</v>
+        <v>57.1</v>
       </c>
       <c r="J15" t="n">
         <v>60.5</v>
@@ -710,31 +710,31 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>44.7</v>
+        <v>44.2</v>
       </c>
       <c r="C16" t="n">
-        <v>47.6</v>
+        <v>47.5</v>
       </c>
       <c r="D16" t="n">
         <v>51.1</v>
       </c>
       <c r="E16" t="n">
-        <v>52.6</v>
+        <v>52.5</v>
       </c>
       <c r="F16" t="n">
-        <v>53.6</v>
+        <v>53.7</v>
       </c>
       <c r="G16" t="n">
-        <v>54.7</v>
+        <v>54.9</v>
       </c>
       <c r="H16" t="n">
-        <v>54.7</v>
+        <v>54.5</v>
       </c>
       <c r="I16" t="n">
-        <v>58.8</v>
+        <v>59.0</v>
       </c>
       <c r="J16" t="n">
-        <v>62.4</v>
+        <v>62.5</v>
       </c>
       <c r="K16" t="n" s="2">
         <v>44768.0</v>
@@ -748,7 +748,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>44.7</v>
+        <v>44.2</v>
       </c>
       <c r="C17" t="n">
         <v>46.2</v>
@@ -757,22 +757,22 @@
         <v>48.7</v>
       </c>
       <c r="E17" t="n">
-        <v>53.4</v>
+        <v>52.9</v>
       </c>
       <c r="F17" t="n">
-        <v>54.5</v>
+        <v>54.3</v>
       </c>
       <c r="G17" t="n">
-        <v>55.4</v>
+        <v>55.5</v>
       </c>
       <c r="H17" t="n">
-        <v>60.0</v>
+        <v>58.2</v>
       </c>
       <c r="I17" t="n">
-        <v>61.9</v>
+        <v>61.6</v>
       </c>
       <c r="J17" t="n">
-        <v>64.0</v>
+        <v>64.2</v>
       </c>
       <c r="K17" t="n" s="2">
         <v>44768.0</v>
@@ -786,31 +786,31 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>41.3</v>
+        <v>41.8</v>
       </c>
       <c r="C18" t="n">
-        <v>44.1</v>
+        <v>44.2</v>
       </c>
       <c r="D18" t="n">
-        <v>46.7</v>
+        <v>47.2</v>
       </c>
       <c r="E18" t="n">
-        <v>51.7</v>
+        <v>51.6</v>
       </c>
       <c r="F18" t="n">
         <v>52.5</v>
       </c>
       <c r="G18" t="n">
-        <v>53.4</v>
+        <v>53.3</v>
       </c>
       <c r="H18" t="n">
-        <v>57.4</v>
+        <v>57.2</v>
       </c>
       <c r="I18" t="n">
-        <v>59.8</v>
+        <v>59.7</v>
       </c>
       <c r="J18" t="n">
-        <v>63.3</v>
+        <v>62.5</v>
       </c>
       <c r="K18" t="n" s="2">
         <v>44768.0</v>
@@ -827,22 +827,22 @@
         <v>47.2</v>
       </c>
       <c r="C19" t="n">
-        <v>48.4</v>
+        <v>48.5</v>
       </c>
       <c r="D19" t="n">
         <v>50.2</v>
       </c>
       <c r="E19" t="n">
-        <v>51.2</v>
+        <v>51.1</v>
       </c>
       <c r="F19" t="n">
         <v>51.8</v>
       </c>
       <c r="G19" t="n">
-        <v>52.5</v>
+        <v>52.7</v>
       </c>
       <c r="H19" t="n">
-        <v>53.3</v>
+        <v>53.1</v>
       </c>
       <c r="I19" t="n">
         <v>54.7</v>
@@ -862,31 +862,31 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>42.0</v>
+        <v>41.8</v>
       </c>
       <c r="C20" t="n">
-        <v>46.2</v>
+        <v>46.3</v>
       </c>
       <c r="D20" t="n">
-        <v>48.9</v>
+        <v>49.7</v>
       </c>
       <c r="E20" t="n">
-        <v>51.1</v>
+        <v>51.2</v>
       </c>
       <c r="F20" t="n">
-        <v>52.0</v>
+        <v>52.2</v>
       </c>
       <c r="G20" t="n">
-        <v>53.3</v>
+        <v>53.7</v>
       </c>
       <c r="H20" t="n">
         <v>54.4</v>
       </c>
       <c r="I20" t="n">
-        <v>57.3</v>
+        <v>57.6</v>
       </c>
       <c r="J20" t="n">
-        <v>62.0</v>
+        <v>64.0</v>
       </c>
       <c r="K20" t="n" s="2">
         <v>44768.0</v>
@@ -900,31 +900,31 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>39.3</v>
+        <v>37.8</v>
       </c>
       <c r="C21" t="n">
-        <v>44.0</v>
+        <v>44.1</v>
       </c>
       <c r="D21" t="n">
-        <v>47.4</v>
+        <v>48.2</v>
       </c>
       <c r="E21" t="n">
-        <v>54.5</v>
+        <v>54.3</v>
       </c>
       <c r="F21" t="n">
-        <v>56.2</v>
+        <v>56.1</v>
       </c>
       <c r="G21" t="n">
-        <v>59.4</v>
+        <v>59.7</v>
       </c>
       <c r="H21" t="n">
-        <v>61.2</v>
+        <v>60.6</v>
       </c>
       <c r="I21" t="n">
-        <v>67.2</v>
+        <v>66.7</v>
       </c>
       <c r="J21" t="n">
-        <v>76.0</v>
+        <v>77.9</v>
       </c>
       <c r="K21" t="n" s="2">
         <v>44768.0</v>
@@ -938,10 +938,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>37.6</v>
+        <v>36.8</v>
       </c>
       <c r="C22" t="n">
-        <v>44.2</v>
+        <v>43.9</v>
       </c>
       <c r="D22" t="n">
         <v>47.7</v>
@@ -950,19 +950,19 @@
         <v>52.0</v>
       </c>
       <c r="F22" t="n">
-        <v>52.9</v>
+        <v>53.0</v>
       </c>
       <c r="G22" t="n">
-        <v>54.9</v>
+        <v>55.2</v>
       </c>
       <c r="H22" t="n">
-        <v>56.9</v>
+        <v>56.6</v>
       </c>
       <c r="I22" t="n">
-        <v>60.4</v>
+        <v>60.9</v>
       </c>
       <c r="J22" t="n">
-        <v>69.0</v>
+        <v>70.4</v>
       </c>
       <c r="K22" t="n" s="2">
         <v>44768.0</v>
@@ -976,31 +976,31 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>43.7</v>
+        <v>43.2</v>
       </c>
       <c r="C23" t="n">
-        <v>47.7</v>
+        <v>47.5</v>
       </c>
       <c r="D23" t="n">
         <v>50.6</v>
       </c>
       <c r="E23" t="n">
-        <v>52.7</v>
+        <v>52.5</v>
       </c>
       <c r="F23" t="n">
         <v>53.5</v>
       </c>
       <c r="G23" t="n">
-        <v>55.1</v>
+        <v>54.8</v>
       </c>
       <c r="H23" t="n">
-        <v>55.7</v>
+        <v>55.3</v>
       </c>
       <c r="I23" t="n">
-        <v>59.0</v>
+        <v>59.1</v>
       </c>
       <c r="J23" t="n">
-        <v>62.3</v>
+        <v>63.1</v>
       </c>
       <c r="K23" t="n" s="2">
         <v>44768.0</v>
@@ -1017,28 +1017,28 @@
         <v>37.8</v>
       </c>
       <c r="C24" t="n">
-        <v>41.3</v>
+        <v>41.6</v>
       </c>
       <c r="D24" t="n">
-        <v>44.2</v>
+        <v>45.2</v>
       </c>
       <c r="E24" t="n">
-        <v>48.3</v>
+        <v>48.1</v>
       </c>
       <c r="F24" t="n">
         <v>49.1</v>
       </c>
       <c r="G24" t="n">
-        <v>50.1</v>
+        <v>50.4</v>
       </c>
       <c r="H24" t="n">
-        <v>53.0</v>
+        <v>52.3</v>
       </c>
       <c r="I24" t="n">
-        <v>56.1</v>
+        <v>55.7</v>
       </c>
       <c r="J24" t="n">
-        <v>59.6</v>
+        <v>60.2</v>
       </c>
       <c r="K24" t="n" s="2">
         <v>45063.0</v>
@@ -1052,28 +1052,28 @@
         <v>14</v>
       </c>
       <c r="B25" t="n">
-        <v>38.0</v>
+        <v>37.8</v>
       </c>
       <c r="C25" t="n">
-        <v>42.3</v>
+        <v>42.5</v>
       </c>
       <c r="D25" t="n">
-        <v>45.7</v>
+        <v>46.2</v>
       </c>
       <c r="E25" t="n">
-        <v>47.8</v>
+        <v>47.5</v>
       </c>
       <c r="F25" t="n">
         <v>48.6</v>
       </c>
       <c r="G25" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="H25" t="n">
         <v>50.1</v>
       </c>
-      <c r="H25" t="n">
-        <v>50.4</v>
-      </c>
       <c r="I25" t="n">
-        <v>54.2</v>
+        <v>54.0</v>
       </c>
       <c r="J25" t="n">
         <v>59.5</v>
@@ -1090,31 +1090,31 @@
         <v>17</v>
       </c>
       <c r="B26" t="n">
-        <v>37.1</v>
+        <v>36.8</v>
       </c>
       <c r="C26" t="n">
-        <v>39.9</v>
+        <v>40.2</v>
       </c>
       <c r="D26" t="n">
-        <v>43.0</v>
+        <v>43.2</v>
       </c>
       <c r="E26" t="n">
-        <v>49.1</v>
+        <v>48.8</v>
       </c>
       <c r="F26" t="n">
-        <v>49.8</v>
+        <v>49.7</v>
       </c>
       <c r="G26" t="n">
         <v>51.0</v>
       </c>
       <c r="H26" t="n">
-        <v>55.5</v>
+        <v>54.6</v>
       </c>
       <c r="I26" t="n">
-        <v>58.5</v>
+        <v>58.1</v>
       </c>
       <c r="J26" t="n">
-        <v>62.1</v>
+        <v>62.6</v>
       </c>
       <c r="K26" t="n" s="2">
         <v>45063.0</v>
@@ -1128,31 +1128,31 @@
         <v>12</v>
       </c>
       <c r="B27" t="n">
-        <v>42.7</v>
+        <v>42.3</v>
       </c>
       <c r="C27" t="n">
-        <v>45.6</v>
+        <v>45.5</v>
       </c>
       <c r="D27" t="n">
-        <v>47.9</v>
+        <v>47.7</v>
       </c>
       <c r="E27" t="n">
-        <v>47.9</v>
+        <v>47.7</v>
       </c>
       <c r="F27" t="n">
         <v>48.8</v>
       </c>
       <c r="G27" t="n">
-        <v>49.8</v>
+        <v>49.7</v>
       </c>
       <c r="H27" t="n">
-        <v>50.0</v>
+        <v>49.4</v>
       </c>
       <c r="I27" t="n">
-        <v>52.0</v>
+        <v>51.9</v>
       </c>
       <c r="J27" t="n">
-        <v>53.7</v>
+        <v>54.2</v>
       </c>
       <c r="K27" t="n" s="2">
         <v>45077.0</v>
@@ -1169,7 +1169,7 @@
         <v>42.3</v>
       </c>
       <c r="C28" t="n">
-        <v>43.5</v>
+        <v>43.6</v>
       </c>
       <c r="D28" t="n">
         <v>45.2</v>
@@ -1181,13 +1181,13 @@
         <v>48.4</v>
       </c>
       <c r="G28" t="n">
-        <v>49.0</v>
+        <v>49.1</v>
       </c>
       <c r="H28" t="n">
-        <v>51.0</v>
+        <v>50.9</v>
       </c>
       <c r="I28" t="n">
-        <v>52.7</v>
+        <v>52.6</v>
       </c>
       <c r="J28" t="n">
         <v>54.1</v>
@@ -1207,10 +1207,10 @@
         <v>38.3</v>
       </c>
       <c r="C29" t="n">
-        <v>40.7</v>
+        <v>40.6</v>
       </c>
       <c r="D29" t="n">
-        <v>43.5</v>
+        <v>43.2</v>
       </c>
       <c r="E29" t="n">
         <v>48.4</v>
@@ -1219,16 +1219,16 @@
         <v>49.3</v>
       </c>
       <c r="G29" t="n">
-        <v>50.2</v>
+        <v>50.1</v>
       </c>
       <c r="H29" t="n">
-        <v>55.3</v>
+        <v>55.1</v>
       </c>
       <c r="I29" t="n">
-        <v>56.8</v>
+        <v>56.9</v>
       </c>
       <c r="J29" t="n">
-        <v>59.2</v>
+        <v>58.9</v>
       </c>
       <c r="K29" t="n" s="2">
         <v>45077.0</v>
@@ -1245,10 +1245,10 @@
         <v>41.3</v>
       </c>
       <c r="C30" t="n">
-        <v>43.8</v>
+        <v>43.7</v>
       </c>
       <c r="D30" t="n">
-        <v>48.4</v>
+        <v>48.2</v>
       </c>
       <c r="E30" t="n">
         <v>48.0</v>
@@ -1257,16 +1257,16 @@
         <v>49.2</v>
       </c>
       <c r="G30" t="n">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
       <c r="H30" t="n">
-        <v>52.2</v>
+        <v>52.3</v>
       </c>
       <c r="I30" t="n">
-        <v>54.0</v>
+        <v>54.2</v>
       </c>
       <c r="J30" t="n">
-        <v>55.7</v>
+        <v>55.9</v>
       </c>
       <c r="K30" t="n" s="2">
         <v>45090.0</v>
@@ -1280,31 +1280,31 @@
         <v>13</v>
       </c>
       <c r="B31" t="n">
-        <v>39.5</v>
+        <v>39.8</v>
       </c>
       <c r="C31" t="n">
-        <v>42.7</v>
+        <v>42.4</v>
       </c>
       <c r="D31" t="n">
         <v>45.7</v>
       </c>
       <c r="E31" t="n">
-        <v>49.5</v>
+        <v>49.6</v>
       </c>
       <c r="F31" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="G31" t="n">
         <v>51.1</v>
       </c>
       <c r="H31" t="n">
-        <v>55.4</v>
+        <v>55.6</v>
       </c>
       <c r="I31" t="n">
-        <v>57.4</v>
+        <v>57.5</v>
       </c>
       <c r="J31" t="n">
-        <v>59.4</v>
+        <v>59.6</v>
       </c>
       <c r="K31" t="n" s="2">
         <v>45090.0</v>
@@ -1321,28 +1321,28 @@
         <v>36.8</v>
       </c>
       <c r="C32" t="n">
-        <v>41.3</v>
+        <v>41.1</v>
       </c>
       <c r="D32" t="n">
-        <v>44.2</v>
+        <v>44.7</v>
       </c>
       <c r="E32" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="F32" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
       <c r="G32" t="n">
-        <v>47.2</v>
+        <v>47.3</v>
       </c>
       <c r="H32" t="n">
-        <v>49.2</v>
+        <v>48.6</v>
       </c>
       <c r="I32" t="n">
         <v>51.6</v>
       </c>
       <c r="J32" t="n">
-        <v>54.3</v>
+        <v>54.2</v>
       </c>
       <c r="K32" t="n" s="2">
         <v>45090.0</v>
@@ -1356,31 +1356,31 @@
         <v>15</v>
       </c>
       <c r="B33" t="n">
-        <v>45.0</v>
+        <v>44.7</v>
       </c>
       <c r="C33" t="n">
-        <v>46.3</v>
+        <v>46.4</v>
       </c>
       <c r="D33" t="n">
-        <v>48.9</v>
+        <v>49.2</v>
       </c>
       <c r="E33" t="n">
-        <v>48.4</v>
+        <v>48.8</v>
       </c>
       <c r="F33" t="n">
-        <v>49.7</v>
+        <v>49.8</v>
       </c>
       <c r="G33" t="n">
-        <v>50.6</v>
+        <v>50.7</v>
       </c>
       <c r="H33" t="n">
-        <v>49.4</v>
+        <v>51.1</v>
       </c>
       <c r="I33" t="n">
-        <v>52.6</v>
+        <v>52.7</v>
       </c>
       <c r="J33" t="n">
-        <v>53.7</v>
+        <v>54.0</v>
       </c>
       <c r="K33" t="n" s="2">
         <v>45090.0</v>
@@ -1394,31 +1394,31 @@
         <v>16</v>
       </c>
       <c r="B34" t="n">
-        <v>42.0</v>
+        <v>41.8</v>
       </c>
       <c r="C34" t="n">
-        <v>45.4</v>
+        <v>45.3</v>
       </c>
       <c r="D34" t="n">
         <v>49.2</v>
       </c>
       <c r="E34" t="n">
-        <v>49.1</v>
+        <v>48.9</v>
       </c>
       <c r="F34" t="n">
         <v>50.1</v>
       </c>
       <c r="G34" t="n">
-        <v>51.1</v>
+        <v>51.0</v>
       </c>
       <c r="H34" t="n">
         <v>51.5</v>
       </c>
       <c r="I34" t="n">
-        <v>54.4</v>
+        <v>54.5</v>
       </c>
       <c r="J34" t="n">
-        <v>56.3</v>
+        <v>57.2</v>
       </c>
       <c r="K34" t="n" s="2">
         <v>45090.0</v>
@@ -1432,31 +1432,31 @@
         <v>17</v>
       </c>
       <c r="B35" t="n">
-        <v>36.8</v>
+        <v>36.3</v>
       </c>
       <c r="C35" t="n">
-        <v>39.4</v>
+        <v>39.2</v>
       </c>
       <c r="D35" t="n">
-        <v>42.7</v>
+        <v>42.3</v>
       </c>
       <c r="E35" t="n">
-        <v>49.1</v>
+        <v>49.3</v>
       </c>
       <c r="F35" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="G35" t="n">
-        <v>51.6</v>
+        <v>51.5</v>
       </c>
       <c r="H35" t="n">
-        <v>58.2</v>
+        <v>57.9</v>
       </c>
       <c r="I35" t="n">
-        <v>60.3</v>
+        <v>60.2</v>
       </c>
       <c r="J35" t="n">
-        <v>62.4</v>
+        <v>63.2</v>
       </c>
       <c r="K35" t="n" s="2">
         <v>45090.0</v>
@@ -1470,31 +1470,31 @@
         <v>18</v>
       </c>
       <c r="B36" t="n">
-        <v>36.5</v>
+        <v>36.3</v>
       </c>
       <c r="C36" t="n">
-        <v>41.0</v>
+        <v>40.4</v>
       </c>
       <c r="D36" t="n">
         <v>45.2</v>
       </c>
       <c r="E36" t="n">
-        <v>44.4</v>
+        <v>44.6</v>
       </c>
       <c r="F36" t="n">
-        <v>46.1</v>
+        <v>45.9</v>
       </c>
       <c r="G36" t="n">
-        <v>47.2</v>
+        <v>47.3</v>
       </c>
       <c r="H36" t="n">
-        <v>48.4</v>
+        <v>48.6</v>
       </c>
       <c r="I36" t="n">
-        <v>50.7</v>
+        <v>51.1</v>
       </c>
       <c r="J36" t="n">
-        <v>52.9</v>
+        <v>53.3</v>
       </c>
       <c r="K36" t="n" s="2">
         <v>45090.0</v>
@@ -1508,13 +1508,13 @@
         <v>19</v>
       </c>
       <c r="B37" t="n">
-        <v>32.1</v>
+        <v>30.4</v>
       </c>
       <c r="C37" t="n">
-        <v>42.3</v>
+        <v>42.2</v>
       </c>
       <c r="D37" t="n">
-        <v>49.0</v>
+        <v>49.2</v>
       </c>
       <c r="E37" t="n">
         <v>47.4</v>
@@ -1523,16 +1523,16 @@
         <v>49.5</v>
       </c>
       <c r="G37" t="n">
-        <v>50.9</v>
+        <v>51.0</v>
       </c>
       <c r="H37" t="n">
-        <v>51.3</v>
+        <v>52.2</v>
       </c>
       <c r="I37" t="n">
-        <v>56.8</v>
+        <v>57.0</v>
       </c>
       <c r="J37" t="n">
-        <v>63.2</v>
+        <v>64.7</v>
       </c>
       <c r="K37" t="n" s="2">
         <v>45090.0</v>
@@ -1546,16 +1546,16 @@
         <v>20</v>
       </c>
       <c r="B38" t="n">
-        <v>36.8</v>
+        <v>36.3</v>
       </c>
       <c r="C38" t="n">
-        <v>38.8</v>
+        <v>38.7</v>
       </c>
       <c r="D38" t="n">
-        <v>40.5</v>
+        <v>40.8</v>
       </c>
       <c r="E38" t="n">
-        <v>49.7</v>
+        <v>49.6</v>
       </c>
       <c r="F38" t="n">
         <v>50.4</v>
@@ -1564,13 +1564,13 @@
         <v>51.3</v>
       </c>
       <c r="H38" t="n">
-        <v>58.3</v>
+        <v>58.2</v>
       </c>
       <c r="I38" t="n">
-        <v>60.4</v>
+        <v>60.5</v>
       </c>
       <c r="J38" t="n">
-        <v>62.1</v>
+        <v>62.8</v>
       </c>
       <c r="K38" t="n" s="2">
         <v>45090.0</v>
@@ -1587,28 +1587,28 @@
         <v>40.8</v>
       </c>
       <c r="C39" t="n">
-        <v>41.8</v>
+        <v>41.9</v>
       </c>
       <c r="D39" t="n">
-        <v>42.7</v>
+        <v>43.2</v>
       </c>
       <c r="E39" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="F39" t="n">
-        <v>50.9</v>
+        <v>50.8</v>
       </c>
       <c r="G39" t="n">
-        <v>51.4</v>
+        <v>51.3</v>
       </c>
       <c r="H39" t="n">
-        <v>57.7</v>
+        <v>57.2</v>
       </c>
       <c r="I39" t="n">
-        <v>58.9</v>
+        <v>58.8</v>
       </c>
       <c r="J39" t="n">
-        <v>60.0</v>
+        <v>60.2</v>
       </c>
       <c r="K39" t="n" s="2">
         <v>45090.0</v>
@@ -1622,31 +1622,31 @@
         <v>22</v>
       </c>
       <c r="B40" t="n">
-        <v>34.8</v>
+        <v>32.9</v>
       </c>
       <c r="C40" t="n">
-        <v>41.5</v>
+        <v>41.2</v>
       </c>
       <c r="D40" t="n">
-        <v>46.7</v>
+        <v>47.2</v>
       </c>
       <c r="E40" t="n">
-        <v>47.5</v>
+        <v>47.0</v>
       </c>
       <c r="F40" t="n">
         <v>48.8</v>
       </c>
       <c r="G40" t="n">
-        <v>50.3</v>
+        <v>50.4</v>
       </c>
       <c r="H40" t="n">
-        <v>53.0</v>
+        <v>52.9</v>
       </c>
       <c r="I40" t="n">
-        <v>56.0</v>
+        <v>56.2</v>
       </c>
       <c r="J40" t="n">
-        <v>60.0</v>
+        <v>61.7</v>
       </c>
       <c r="K40" t="n" s="2">
         <v>45090.0</v>
@@ -1660,31 +1660,31 @@
         <v>12</v>
       </c>
       <c r="B41" t="n">
-        <v>38.8</v>
+        <v>37.8</v>
       </c>
       <c r="C41" t="n">
-        <v>44.2</v>
+        <v>43.7</v>
       </c>
       <c r="D41" t="n">
         <v>49.2</v>
       </c>
       <c r="E41" t="n">
-        <v>47.9</v>
+        <v>47.7</v>
       </c>
       <c r="F41" t="n">
-        <v>49.6</v>
+        <v>49.5</v>
       </c>
       <c r="G41" t="n">
         <v>51.0</v>
       </c>
       <c r="H41" t="n">
-        <v>51.2</v>
+        <v>51.0</v>
       </c>
       <c r="I41" t="n">
-        <v>54.1</v>
+        <v>54.3</v>
       </c>
       <c r="J41" t="n">
-        <v>57.8</v>
+        <v>58.0</v>
       </c>
       <c r="K41" t="n" s="2">
         <v>45130.0</v>
@@ -1698,31 +1698,31 @@
         <v>13</v>
       </c>
       <c r="B42" t="n">
-        <v>42.7</v>
+        <v>42.3</v>
       </c>
       <c r="C42" t="n">
-        <v>44.5</v>
+        <v>44.4</v>
       </c>
       <c r="D42" t="n">
-        <v>46.5</v>
+        <v>46.2</v>
       </c>
       <c r="E42" t="n">
-        <v>50.0</v>
+        <v>49.8</v>
       </c>
       <c r="F42" t="n">
-        <v>50.5</v>
+        <v>50.4</v>
       </c>
       <c r="G42" t="n">
-        <v>50.8</v>
+        <v>50.9</v>
       </c>
       <c r="H42" t="n">
-        <v>54.4</v>
+        <v>54.2</v>
       </c>
       <c r="I42" t="n">
-        <v>55.7</v>
+        <v>55.8</v>
       </c>
       <c r="J42" t="n">
-        <v>57.1</v>
+        <v>57.2</v>
       </c>
       <c r="K42" t="n" s="2">
         <v>45130.0</v>
@@ -1736,31 +1736,31 @@
         <v>14</v>
       </c>
       <c r="B43" t="n">
-        <v>39.0</v>
+        <v>39.3</v>
       </c>
       <c r="C43" t="n">
-        <v>43.8</v>
+        <v>44.2</v>
       </c>
       <c r="D43" t="n">
-        <v>47.9</v>
+        <v>48.2</v>
       </c>
       <c r="E43" t="n">
-        <v>48.7</v>
+        <v>48.6</v>
       </c>
       <c r="F43" t="n">
-        <v>49.7</v>
+        <v>49.8</v>
       </c>
       <c r="G43" t="n">
         <v>50.8</v>
       </c>
       <c r="H43" t="n">
-        <v>52.8</v>
+        <v>52.9</v>
       </c>
       <c r="I43" t="n">
-        <v>55.4</v>
+        <v>55.1</v>
       </c>
       <c r="J43" t="n">
-        <v>58.7</v>
+        <v>58.5</v>
       </c>
       <c r="K43" t="n" s="2">
         <v>45130.0</v>
@@ -1774,19 +1774,19 @@
         <v>15</v>
       </c>
       <c r="B44" t="n">
-        <v>37.3</v>
+        <v>38.8</v>
       </c>
       <c r="C44" t="n">
-        <v>45.1</v>
+        <v>45.5</v>
       </c>
       <c r="D44" t="n">
-        <v>49.2</v>
+        <v>49.7</v>
       </c>
       <c r="E44" t="n">
-        <v>49.8</v>
+        <v>49.9</v>
       </c>
       <c r="F44" t="n">
-        <v>51.0</v>
+        <v>51.1</v>
       </c>
       <c r="G44" t="n">
         <v>51.9</v>
@@ -1795,10 +1795,10 @@
         <v>53.0</v>
       </c>
       <c r="I44" t="n">
-        <v>56.0</v>
+        <v>55.8</v>
       </c>
       <c r="J44" t="n">
-        <v>60.7</v>
+        <v>61.0</v>
       </c>
       <c r="K44" t="n" s="2">
         <v>45130.0</v>
@@ -1812,7 +1812,7 @@
         <v>16</v>
       </c>
       <c r="B45" t="n">
-        <v>39.0</v>
+        <v>38.8</v>
       </c>
       <c r="C45" t="n">
         <v>42.7</v>
@@ -1821,22 +1821,22 @@
         <v>49.2</v>
       </c>
       <c r="E45" t="n">
-        <v>50.4</v>
+        <v>50.3</v>
       </c>
       <c r="F45" t="n">
-        <v>51.7</v>
+        <v>51.6</v>
       </c>
       <c r="G45" t="n">
-        <v>53.6</v>
+        <v>53.4</v>
       </c>
       <c r="H45" t="n">
         <v>51.8</v>
       </c>
       <c r="I45" t="n">
-        <v>59.8</v>
+        <v>59.6</v>
       </c>
       <c r="J45" t="n">
-        <v>63.8</v>
+        <v>64.2</v>
       </c>
       <c r="K45" t="n" s="2">
         <v>45130.0</v>
@@ -1853,28 +1853,28 @@
         <v>37.8</v>
       </c>
       <c r="C46" t="n">
-        <v>41.4</v>
+        <v>41.2</v>
       </c>
       <c r="D46" t="n">
-        <v>45.2</v>
+        <v>44.7</v>
       </c>
       <c r="E46" t="n">
         <v>49.7</v>
       </c>
       <c r="F46" t="n">
-        <v>50.7</v>
+        <v>50.6</v>
       </c>
       <c r="G46" t="n">
-        <v>51.7</v>
+        <v>51.6</v>
       </c>
       <c r="H46" t="n">
-        <v>55.9</v>
+        <v>56.4</v>
       </c>
       <c r="I46" t="n">
         <v>59.1</v>
       </c>
       <c r="J46" t="n">
-        <v>62.3</v>
+        <v>62.4</v>
       </c>
       <c r="K46" t="n" s="2">
         <v>45130.0</v>
@@ -1888,13 +1888,13 @@
         <v>18</v>
       </c>
       <c r="B47" t="n">
-        <v>34.6</v>
+        <v>35.3</v>
       </c>
       <c r="C47" t="n">
-        <v>39.7</v>
+        <v>39.9</v>
       </c>
       <c r="D47" t="n">
-        <v>44.3</v>
+        <v>45.7</v>
       </c>
       <c r="E47" t="n">
         <v>46.1</v>
@@ -1903,16 +1903,16 @@
         <v>47.6</v>
       </c>
       <c r="G47" t="n">
-        <v>48.8</v>
+        <v>49.2</v>
       </c>
       <c r="H47" t="n">
-        <v>52.1</v>
+        <v>51.5</v>
       </c>
       <c r="I47" t="n">
-        <v>54.7</v>
+        <v>54.5</v>
       </c>
       <c r="J47" t="n">
-        <v>57.3</v>
+        <v>57.6</v>
       </c>
       <c r="K47" t="n" s="2">
         <v>45130.0</v>
@@ -1929,25 +1929,25 @@
         <v>45.7</v>
       </c>
       <c r="C48" t="n">
-        <v>49.0</v>
+        <v>49.1</v>
       </c>
       <c r="D48" t="n">
         <v>52.1</v>
       </c>
       <c r="E48" t="n">
-        <v>52.0</v>
+        <v>52.3</v>
       </c>
       <c r="F48" t="n">
         <v>53.6</v>
       </c>
       <c r="G48" t="n">
-        <v>55.3</v>
+        <v>55.6</v>
       </c>
       <c r="H48" t="n">
         <v>53.6</v>
       </c>
       <c r="I48" t="n">
-        <v>57.0</v>
+        <v>56.9</v>
       </c>
       <c r="J48" t="n">
         <v>61.2</v>
@@ -1964,16 +1964,16 @@
         <v>20</v>
       </c>
       <c r="B49" t="n">
-        <v>42.0</v>
+        <v>41.3</v>
       </c>
       <c r="C49" t="n">
-        <v>45.1</v>
+        <v>44.8</v>
       </c>
       <c r="D49" t="n">
-        <v>48.2</v>
+        <v>48.7</v>
       </c>
       <c r="E49" t="n">
-        <v>52.7</v>
+        <v>52.8</v>
       </c>
       <c r="F49" t="n">
         <v>54.3</v>
@@ -1982,13 +1982,13 @@
         <v>55.7</v>
       </c>
       <c r="H49" t="n">
-        <v>59.7</v>
+        <v>59.4</v>
       </c>
       <c r="I49" t="n">
-        <v>62.1</v>
+        <v>62.3</v>
       </c>
       <c r="J49" t="n">
-        <v>64.6</v>
+        <v>65.3</v>
       </c>
       <c r="K49" t="n" s="2">
         <v>45130.0</v>
@@ -2002,31 +2002,31 @@
         <v>21</v>
       </c>
       <c r="B50" t="n">
-        <v>41.0</v>
+        <v>40.8</v>
       </c>
       <c r="C50" t="n">
-        <v>42.9</v>
+        <v>42.8</v>
       </c>
       <c r="D50" t="n">
         <v>44.7</v>
       </c>
       <c r="E50" t="n">
-        <v>50.2</v>
+        <v>50.6</v>
       </c>
       <c r="F50" t="n">
-        <v>51.4</v>
+        <v>51.5</v>
       </c>
       <c r="G50" t="n">
-        <v>52.2</v>
+        <v>52.4</v>
       </c>
       <c r="H50" t="n">
-        <v>55.6</v>
+        <v>56.1</v>
       </c>
       <c r="I50" t="n">
-        <v>58.8</v>
+        <v>59.0</v>
       </c>
       <c r="J50" t="n">
-        <v>61.0</v>
+        <v>61.2</v>
       </c>
       <c r="K50" t="n" s="2">
         <v>45130.0</v>
@@ -2040,31 +2040,31 @@
         <v>22</v>
       </c>
       <c r="B51" t="n">
-        <v>37.6</v>
+        <v>37.3</v>
       </c>
       <c r="C51" t="n">
-        <v>43.6</v>
+        <v>43.9</v>
       </c>
       <c r="D51" t="n">
-        <v>50.2</v>
+        <v>50.6</v>
       </c>
       <c r="E51" t="n">
-        <v>49.9</v>
+        <v>49.8</v>
       </c>
       <c r="F51" t="n">
         <v>51.2</v>
       </c>
       <c r="G51" t="n">
-        <v>52.5</v>
+        <v>52.7</v>
       </c>
       <c r="H51" t="n">
-        <v>54.6</v>
+        <v>54.4</v>
       </c>
       <c r="I51" t="n">
-        <v>58.3</v>
+        <v>58.2</v>
       </c>
       <c r="J51" t="n">
-        <v>63.3</v>
+        <v>63.0</v>
       </c>
       <c r="K51" t="n" s="2">
         <v>45130.0</v>
@@ -2078,31 +2078,31 @@
         <v>12</v>
       </c>
       <c r="B52" t="n">
-        <v>32.1</v>
+        <v>30.4</v>
       </c>
       <c r="C52" t="n">
-        <v>42.1</v>
+        <v>41.2</v>
       </c>
       <c r="D52" t="n">
-        <v>48.2</v>
+        <v>47.7</v>
       </c>
       <c r="E52" t="n">
-        <v>44.4</v>
+        <v>44.0</v>
       </c>
       <c r="F52" t="n">
-        <v>47.3</v>
+        <v>47.0</v>
       </c>
       <c r="G52" t="n">
-        <v>49.4</v>
+        <v>49.3</v>
       </c>
       <c r="H52" t="n">
-        <v>49.3</v>
+        <v>49.6</v>
       </c>
       <c r="I52" t="n">
-        <v>52.6</v>
+        <v>53.0</v>
       </c>
       <c r="J52" t="n">
-        <v>56.8</v>
+        <v>58.4</v>
       </c>
       <c r="K52" t="n" s="2">
         <v>45180.0</v>
@@ -2116,19 +2116,19 @@
         <v>13</v>
       </c>
       <c r="B53" t="n">
-        <v>43.7</v>
+        <v>43.2</v>
       </c>
       <c r="C53" t="n">
-        <v>47.3</v>
+        <v>47.4</v>
       </c>
       <c r="D53" t="n">
         <v>50.2</v>
       </c>
       <c r="E53" t="n">
-        <v>51.9</v>
+        <v>51.8</v>
       </c>
       <c r="F53" t="n">
-        <v>52.4</v>
+        <v>52.5</v>
       </c>
       <c r="G53" t="n">
         <v>53.0</v>
@@ -2140,7 +2140,7 @@
         <v>57.0</v>
       </c>
       <c r="J53" t="n">
-        <v>59.9</v>
+        <v>60.6</v>
       </c>
       <c r="K53" t="n" s="2">
         <v>45180.0</v>
@@ -2154,31 +2154,31 @@
         <v>14</v>
       </c>
       <c r="B54" t="n">
-        <v>28.4</v>
+        <v>27.4</v>
       </c>
       <c r="C54" t="n">
-        <v>38.4</v>
+        <v>38.6</v>
       </c>
       <c r="D54" t="n">
-        <v>44.0</v>
+        <v>45.2</v>
       </c>
       <c r="E54" t="n">
         <v>44.2</v>
       </c>
       <c r="F54" t="n">
-        <v>46.4</v>
+        <v>46.5</v>
       </c>
       <c r="G54" t="n">
         <v>48.3</v>
       </c>
       <c r="H54" t="n">
-        <v>51.9</v>
+        <v>50.7</v>
       </c>
       <c r="I54" t="n">
-        <v>54.8</v>
+        <v>54.6</v>
       </c>
       <c r="J54" t="n">
-        <v>60.1</v>
+        <v>60.4</v>
       </c>
       <c r="K54" t="n" s="2">
         <v>45180.0</v>
@@ -2192,31 +2192,31 @@
         <v>15</v>
       </c>
       <c r="B55" t="n">
-        <v>45.7</v>
+        <v>45.2</v>
       </c>
       <c r="C55" t="n">
-        <v>47.6</v>
+        <v>47.5</v>
       </c>
       <c r="D55" t="n">
         <v>50.2</v>
       </c>
       <c r="E55" t="n">
-        <v>51.3</v>
+        <v>51.4</v>
       </c>
       <c r="F55" t="n">
         <v>52.0</v>
       </c>
       <c r="G55" t="n">
-        <v>52.7</v>
+        <v>52.5</v>
       </c>
       <c r="H55" t="n">
-        <v>54.1</v>
+        <v>54.3</v>
       </c>
       <c r="I55" t="n">
-        <v>56.0</v>
+        <v>56.1</v>
       </c>
       <c r="J55" t="n">
-        <v>58.1</v>
+        <v>58.4</v>
       </c>
       <c r="K55" t="n" s="2">
         <v>45180.0</v>
@@ -2233,28 +2233,28 @@
         <v>45.2</v>
       </c>
       <c r="C56" t="n">
-        <v>47.7</v>
+        <v>47.8</v>
       </c>
       <c r="D56" t="n">
-        <v>50.2</v>
+        <v>50.6</v>
       </c>
       <c r="E56" t="n">
         <v>50.4</v>
       </c>
       <c r="F56" t="n">
-        <v>51.2</v>
+        <v>51.3</v>
       </c>
       <c r="G56" t="n">
-        <v>52.1</v>
+        <v>52.3</v>
       </c>
       <c r="H56" t="n">
-        <v>52.4</v>
+        <v>52.5</v>
       </c>
       <c r="I56" t="n">
         <v>54.4</v>
       </c>
       <c r="J56" t="n">
-        <v>56.7</v>
+        <v>56.5</v>
       </c>
       <c r="K56" t="n" s="2">
         <v>45180.0</v>
@@ -2268,7 +2268,7 @@
         <v>17</v>
       </c>
       <c r="B57" t="n">
-        <v>40.3</v>
+        <v>39.3</v>
       </c>
       <c r="C57" t="n">
         <v>42.5</v>
@@ -2277,22 +2277,22 @@
         <v>44.7</v>
       </c>
       <c r="E57" t="n">
-        <v>49.4</v>
+        <v>49.2</v>
       </c>
       <c r="F57" t="n">
-        <v>50.2</v>
+        <v>50.1</v>
       </c>
       <c r="G57" t="n">
         <v>51.0</v>
       </c>
       <c r="H57" t="n">
-        <v>54.8</v>
+        <v>54.7</v>
       </c>
       <c r="I57" t="n">
-        <v>56.8</v>
+        <v>56.7</v>
       </c>
       <c r="J57" t="n">
-        <v>59.5</v>
+        <v>59.3</v>
       </c>
       <c r="K57" t="n" s="2">
         <v>45180.0</v>
@@ -2309,28 +2309,28 @@
         <v>23.0</v>
       </c>
       <c r="C58" t="n">
-        <v>27.5</v>
+        <v>27.8</v>
       </c>
       <c r="D58" t="n">
-        <v>42.0</v>
+        <v>42.7</v>
       </c>
       <c r="E58" t="n">
-        <v>37.6</v>
+        <v>37.4</v>
       </c>
       <c r="F58" t="n">
-        <v>41.7</v>
+        <v>41.6</v>
       </c>
       <c r="G58" t="n">
-        <v>45.0</v>
+        <v>45.7</v>
       </c>
       <c r="H58" t="n">
-        <v>50.6</v>
+        <v>49.0</v>
       </c>
       <c r="I58" t="n">
-        <v>56.3</v>
+        <v>55.9</v>
       </c>
       <c r="J58" t="n">
-        <v>63.0</v>
+        <v>62.4</v>
       </c>
       <c r="K58" t="n" s="2">
         <v>45180.0</v>
@@ -2344,31 +2344,31 @@
         <v>19</v>
       </c>
       <c r="B59" t="n">
-        <v>29.2</v>
+        <v>28.4</v>
       </c>
       <c r="C59" t="n">
-        <v>39.8</v>
+        <v>41.0</v>
       </c>
       <c r="D59" t="n">
-        <v>50.4</v>
+        <v>50.6</v>
       </c>
       <c r="E59" t="n">
-        <v>50.2</v>
+        <v>50.1</v>
       </c>
       <c r="F59" t="n">
-        <v>52.1</v>
+        <v>52.2</v>
       </c>
       <c r="G59" t="n">
-        <v>53.6</v>
+        <v>53.7</v>
       </c>
       <c r="H59" t="n">
-        <v>54.8</v>
+        <v>54.2</v>
       </c>
       <c r="I59" t="n">
-        <v>61.5</v>
+        <v>60.9</v>
       </c>
       <c r="J59" t="n">
-        <v>68.6</v>
+        <v>69.7</v>
       </c>
       <c r="K59" t="n" s="2">
         <v>45180.0</v>
@@ -2382,7 +2382,7 @@
         <v>20</v>
       </c>
       <c r="B60" t="n">
-        <v>41.8</v>
+        <v>41.7</v>
       </c>
       <c r="C60" t="n">
         <v>43.5</v>
@@ -2397,13 +2397,13 @@
         <v>52.2</v>
       </c>
       <c r="G60" t="n">
-        <v>52.7</v>
+        <v>52.9</v>
       </c>
       <c r="H60" t="n">
-        <v>57.8</v>
+        <v>58.4</v>
       </c>
       <c r="I60" t="n">
-        <v>60.3</v>
+        <v>60.2</v>
       </c>
       <c r="J60" t="n">
         <v>62.1</v>
@@ -2420,31 +2420,31 @@
         <v>21</v>
       </c>
       <c r="B61" t="n">
-        <v>43.0</v>
+        <v>42.7</v>
       </c>
       <c r="C61" t="n">
-        <v>44.2</v>
+        <v>44.1</v>
       </c>
       <c r="D61" t="n">
-        <v>45.7</v>
+        <v>45.2</v>
       </c>
       <c r="E61" t="n">
-        <v>50.1</v>
+        <v>50.0</v>
       </c>
       <c r="F61" t="n">
-        <v>50.7</v>
+        <v>50.6</v>
       </c>
       <c r="G61" t="n">
         <v>51.3</v>
       </c>
       <c r="H61" t="n">
-        <v>54.5</v>
+        <v>54.6</v>
       </c>
       <c r="I61" t="n">
-        <v>56.2</v>
+        <v>56.3</v>
       </c>
       <c r="J61" t="n">
-        <v>57.3</v>
+        <v>57.8</v>
       </c>
       <c r="K61" t="n" s="2">
         <v>45180.0</v>
@@ -2461,28 +2461,28 @@
         <v>23.0</v>
       </c>
       <c r="C62" t="n">
-        <v>34.0</v>
+        <v>33.3</v>
       </c>
       <c r="D62" t="n">
-        <v>51.5</v>
+        <v>50.9</v>
       </c>
       <c r="E62" t="n">
         <v>43.7</v>
       </c>
       <c r="F62" t="n">
-        <v>48.6</v>
+        <v>48.3</v>
       </c>
       <c r="G62" t="n">
-        <v>52.9</v>
+        <v>52.6</v>
       </c>
       <c r="H62" t="n">
-        <v>54.0</v>
+        <v>53.9</v>
       </c>
       <c r="I62" t="n">
-        <v>65.7</v>
+        <v>65.8</v>
       </c>
       <c r="J62" t="n">
-        <v>86.4</v>
+        <v>85.7</v>
       </c>
       <c r="K62" t="n" s="2">
         <v>45180.0</v>

</xml_diff>